<commit_message>
Updated Excel file with manual test results
</commit_message>
<xml_diff>
--- a/IT23361522_Assignment 1 - Test cases.xlsx
+++ b/IT23361522_Assignment 1 - Test cases.xlsx
@@ -398,16 +398,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H51"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="60.83203125" customWidth="1"/>
-    <col min="4" max="4" width="60.83203125" customWidth="1"/>
-    <col min="5" max="5" width="60.83203125" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" customWidth="1"/>
-    <col min="7" max="7" width="50.83203125" customWidth="1"/>
-    <col min="8" max="8" width="80.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -449,10 +439,10 @@
         <v>අද school ගියනවා ද?</v>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>අද school ගියනවා ද?</v>
       </c>
       <c r="F2" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G2" t="str">
         <v>Question forms</v>
@@ -475,10 +465,10 @@
         <v>මම දන්නේ නා ඔය කොහෙද ගියේ කියලා. අපි හෙට යමුද නැත්නම් අවුරුද්ද වාගේ කරන්නෝ?</v>
       </c>
       <c r="E3" t="str">
-        <v/>
+        <v>මම දන්නේ නා ඔය කොහෙද ගියේ කියලා. අපි හෙට යමුද නැත්නම් අවුරුද්ද වාගේ කරන්නෝ?</v>
       </c>
       <c r="F3" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G3" t="str">
         <v>Question forms; Inputs with Punctuation Marks</v>
@@ -501,10 +491,10 @@
         <v>ඔය API එකේ documentation එකේ බලලා ද? මම එන්නේ ඕනේ නම් ticket එකක් ගන්නද?</v>
       </c>
       <c r="E4" t="str">
-        <v/>
+        <v>ඔය API එකේ documentation එකේ බලලා ද? මම එන්නේ ඕනේ නම් ticket එකක් ගන්නද?</v>
       </c>
       <c r="F4" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G4" t="str">
         <v>Question forms; English Digital Terms in Singlish</v>
@@ -527,10 +517,10 @@
         <v>වහාම ගෙදර යන්නේ! එපා ඉන්නේ.</v>
       </c>
       <c r="E5" t="str">
-        <v/>
+        <v>වහාම ගෙදර යන්නේ! එපා ඉන්නේ.</v>
       </c>
       <c r="F5" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G5" t="str">
         <v>Command forms; Inputs with Punctuation Marks</v>
@@ -553,10 +543,10 @@
         <v>ඒකා කරන්නම් කියලා කියන්නේ එපා. මම කියනවා එහෙම කරන්නේ. හදිල්ලා දන් එන්නකෝ මචන්.</v>
       </c>
       <c r="E6" t="str">
-        <v/>
+        <v>ඒකා කරන්නම් කියලා කියන්නේ එපා. මම කියනවා එහෙම කරන්නේ. හදිල්ලා දන් එන්නකෝ මචන්.</v>
       </c>
       <c r="F6" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G6" t="str">
         <v>Command forms; Inputs with Slang and Casual Phrasing</v>
@@ -579,10 +569,10 @@
         <v>කොහොමද බ්‍රෝ? සුද්ද ද ඉන්නේ?</v>
       </c>
       <c r="E7" t="str">
-        <v/>
+        <v>කොහොමද බ්රෝ? සුද්ද ද ඉන්නේ?</v>
       </c>
       <c r="F7" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G7" t="str">
         <v>Greetings; Inputs with Slang and Casual Phrasing</v>
@@ -605,10 +595,10 @@
         <v>මල්ලි! ගොඩක් දවසක් පස්සේ කෙතුවා නේ. කොහොමද ඉන්නේ ඔය? හොඳ වෙලා තිෙනවා වාගේ පෙනෙවා.</v>
       </c>
       <c r="E8" t="str">
-        <v/>
+        <v>මල්ලි! ගොඩක් දවසක් පස්සේ කෙතුවා නේ. කොහොමද ඉන්නේ ඔය? හොඳ වෙලා තිෙනවා වාගේ පෙනෙවා.</v>
       </c>
       <c r="F8" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G8" t="str">
         <v>Greetings; Inputs with Punctuation Marks</v>
@@ -631,10 +621,10 @@
         <v>කරුණාකරා මෙකා පොඩ්ඩක් බලන්නේ පුළුවන්ද?</v>
       </c>
       <c r="E9" t="str">
-        <v/>
+        <v>කරුණාකරා මෙකා පොඩ්ඩක් බලන්නේ පුළුවන්ද?</v>
       </c>
       <c r="F9" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G9" t="str">
         <v>Requests</v>
@@ -657,10 +647,10 @@
         <v>මම ඔබ කියනවා, ඔය හෙට meeting එකේදී Zoom link එකේ එවන්නේ පුළුවන්ද? මම office එකේ ඉන්නවා හදිස්සියේ.</v>
       </c>
       <c r="E10" t="str">
-        <v/>
+        <v>මම ඔබ කියනවා, ඔය හෙට meeting එකේදී Zoom link එකේ එවන්නේ පුළුවන්ද? මම office එකේ ඉන්නවා හදිස්සියේ.</v>
       </c>
       <c r="F10" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G10" t="str">
         <v>Requests; Platform/App Names in Singlish; Isolated English Word Insertions in Singlish</v>
@@ -683,10 +673,10 @@
         <v>අනේ හරි අයිේ. මම ඒකා කරන්නම්.</v>
       </c>
       <c r="E11" t="str">
-        <v/>
+        <v>අනේ හරි අයිේ. මම ඒකා කරන්නම්.</v>
       </c>
       <c r="F11" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G11" t="str">
         <v>Responses</v>
@@ -709,10 +699,10 @@
         <v>නැතනේ මම දන්නේ. ඒත් ඔය කියනවා නම් ඒකා කරන්නේ. මම හිතුව කරන්නේ ඒත් බැලුවේ නාහා.</v>
       </c>
       <c r="E12" t="str">
-        <v/>
+        <v>නැතනේ මම දන්නේ. ඒත් ඔය කියනවා නම් ඒකා කරන්නේ. මම හිතුව කරන්නේ ඒත් බැලුවේ නාහා.</v>
       </c>
       <c r="F12" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G12" t="str">
         <v>Responses; Inputs with Punctuation Marks</v>
@@ -735,10 +725,10 @@
         <v>බොරු බොරු කතා කියන්නේ එපා.</v>
       </c>
       <c r="E13" t="str">
-        <v/>
+        <v>බොරු බොරු කතා කියන්නේ එපා.</v>
       </c>
       <c r="F13" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G13" t="str">
         <v>Repeated Words; Command forms</v>
@@ -761,10 +751,10 @@
         <v>හරි හරි මම එන්නම්. ගොඩක් ගොඩක් වාගේ ඉන්නවා කියලානේ. පොඩ්ඩක් පොඩ්ඩක් කරාකරාලා මම ඒකා හදාගන්නම්.</v>
       </c>
       <c r="E14" t="str">
-        <v/>
+        <v>හරි හරි මම එන්නම්. ගොඩක් ගොඩක් වාගේ ඉන්නවා කියලානේ. පොඩ්ඩක් පොඩ්ඩක් කරාකරාලා මම ඒකා හදාගන්නම්.</v>
       </c>
       <c r="F14" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G14" t="str">
         <v>Repeated Words</v>
@@ -787,10 +777,10 @@
         <v>අනේ! ඔය එනවාද... නේ?</v>
       </c>
       <c r="E15" t="str">
-        <v/>
+        <v>අනේ! ඔය එනවාද... නේ?</v>
       </c>
       <c r="F15" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G15" t="str">
         <v>Inputs with Punctuation Marks; Responses</v>
@@ -813,10 +803,10 @@
         <v>මම කියනවා, ඔය දන්නා ද මෙකා? හදන්නේ නේ... ඒත් හරි කරන්නේ ඕනේ, නේ! මම ඒකා බලාමු.</v>
       </c>
       <c r="E16" t="str">
-        <v/>
+        <v>මම කියනවා, ඔය දන්නා ද මෙකා? හදන්නේ නේ... ඒත් හරි කරන්නේ ඕනේ, නේ! මම ඒකා බලාමු.</v>
       </c>
       <c r="F16" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G16" t="str">
         <v>Inputs with Punctuation Marks; Question forms</v>
@@ -839,10 +829,10 @@
         <v>මේ එකේ හොඳ නේ මචන්?</v>
       </c>
       <c r="E17" t="str">
-        <v/>
+        <v>මේ එකේ හොඳ නේ මචන්?</v>
       </c>
       <c r="F17" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G17" t="str">
         <v>Romanization / Spelling Variants; Inputs with Slang and Casual Phrasing</v>
@@ -865,10 +855,10 @@
         <v>මං ඔයාට පස්සේ එන්නම් කියලා කිව්වා. ඒත් ඔයාට බලාගෙන ඉන්නේ නේ? මංගෙ ගෙදර ඇහුවොත් එනවා නම්.</v>
       </c>
       <c r="E18" t="str">
-        <v/>
+        <v>මං ඔයාට පස්සේ එන්නම් කියලා කිව්වා. ඒත් ඔයාට බලාගෙන ඉන්නේ නේ? මංගෙ ගෙදර ඇහුවොත් එනවා නම්.</v>
       </c>
       <c r="F18" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G18" t="str">
         <v>Romanization / Spelling Variants</v>
@@ -891,10 +881,10 @@
         <v>lunch කරන්නේ යමු නේ?</v>
       </c>
       <c r="E19" t="str">
-        <v/>
+        <v>lunch කරන්නේ යමු නේ?</v>
       </c>
       <c r="F19" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G19" t="str">
         <v>Isolated English Word Insertions in Singlish; Question forms</v>
@@ -917,10 +907,10 @@
         <v>මම අද project එකේ finish කරන්නම් කියලා හිතුව ඒත් deadline එකේ miss උනා නිසා manager කියනවා extension එකක් ගන්නේ කියලා.</v>
       </c>
       <c r="E20" t="str">
-        <v/>
+        <v>මම අද project එකේ finish කරන්නම් කියලා හිතුව ඒත් deadline එකේ miss උනා නිසා manager කියනවා extension එකක් ගන්නේ කියලා.</v>
       </c>
       <c r="F20" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G20" t="str">
         <v>Isolated English Word Insertions in Singlish</v>
@@ -943,10 +933,10 @@
         <v>මම කියනවා out of stock වෙලා තිෙනවා ඒත් just in case order කරන්නේ හිතුව නේ.</v>
       </c>
       <c r="E21" t="str">
-        <v/>
+        <v>මම කියනවා out of stock වෙලා තිෙනවා ඒත් just in case order කරන්නේ හිතුව නේ.</v>
       </c>
       <c r="F21" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G21" t="str">
         <v>Multi-Word English Phrases in Singlish; Isolated English Word Insertions in Singlish</v>
@@ -969,10 +959,10 @@
         <v>ඔය දන්නවා ද free of charge ලැබෙන බව? ඒත් terms and conditions බලන්නේ ඕනේ කියලානේ. as soon as possible submit කරන්නේ.</v>
       </c>
       <c r="E22" t="str">
-        <v/>
+        <v>ඔය දන්නවා ද free of charge ලැබෙන බව? ඒත් terms and conditions බලන්නේ ඕනේ කියලානේ. as soon as possible submit කරන්නේ.</v>
       </c>
       <c r="F22" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G22" t="str">
         <v>Multi-Word English Phrases in Singlish; Question forms; Inputs with Punctuation Marks</v>
@@ -995,10 +985,10 @@
         <v>download link එකේ පෙන්නන්නේ.</v>
       </c>
       <c r="E23" t="str">
-        <v/>
+        <v>download link එකේ පෙන්නන්නේ.</v>
       </c>
       <c r="F23" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G23" t="str">
         <v>English Digital Terms in Singlish; Requests</v>
@@ -1021,10 +1011,10 @@
         <v>ඔය account එකේ login කරන්නේ පුළුවන් ඒත් password reset කරන්නේ ඕනේ කියන්නේ කොච්චරද? email එකේ confirm වෙවිද?</v>
       </c>
       <c r="E24" t="str">
-        <v/>
+        <v>ඔය account එකේ login කරන්නේ පුළුවන් ඒත් password reset කරන්නේ ඕනේ කියන්නේ කොච්චරද? email එකේ confirm වෙවිද?</v>
       </c>
       <c r="F24" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G24" t="str">
         <v>English Digital Terms in Singlish; Question forms</v>
@@ -1047,10 +1037,10 @@
         <v>Viber එකෙන් message එකක් එව.</v>
       </c>
       <c r="E25" t="str">
-        <v/>
+        <v>Viber එකෙන් message එකක් එව.</v>
       </c>
       <c r="F25" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G25" t="str">
         <v>Platform/App Names in Singlish; Requests</v>
@@ -1073,10 +1063,10 @@
         <v>මම Facebook එකේ post එකක් දාම්ම අපි Instagram වලට share කරන්නම් කියලා කිව්වා. TikTok එකේ trend එකේ බල්ලකෝ.</v>
       </c>
       <c r="E26" t="str">
-        <v/>
+        <v>මම Facebook එකේ post එකක් දාම්ම අපි Instagram වලට share කරන්නම් කියලා කිව්වා. TikTok එකේ trend එකේ බල්ලකෝ.</v>
       </c>
       <c r="F26" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G26" t="str">
         <v>Platform/App Names in Singlish; Isolated English Word Insertions in Singlish</v>
@@ -1099,10 +1089,10 @@
         <v>ASAP කරන්නම් ok ද?</v>
       </c>
       <c r="E27" t="str">
-        <v/>
+        <v>ASAP කරන්නම් ok ද?</v>
       </c>
       <c r="F27" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G27" t="str">
         <v>English Abbreviations/Acronyms in Singlish; Question forms</v>
@@ -1125,10 +1115,10 @@
         <v>ඔය CV එකේ update කරලාද? HR කියනවා ASAP submit කරන්නේ කියලා. ඒත් DOB සහ NIC එකේ හරිද check කරන්නේ.</v>
       </c>
       <c r="E28" t="str">
-        <v/>
+        <v>ඔය CV එකේ update කරලාද? HR කියනවා ASAP submit කරන්නේ කියලා. ඒත් DOB සහ NIC එකේ හරිද check කරන්නේ.</v>
       </c>
       <c r="F28" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G28" t="str">
         <v>English Abbreviations/Acronyms in Singlish; Question forms; Isolated English Word Insertions in Singlish</v>
@@ -1151,10 +1141,10 @@
         <v>prof එකෙන් lab assignment එකක් තිෙනවා.</v>
       </c>
       <c r="E29" t="str">
-        <v/>
+        <v>prof එකෙන් lab assignment එකක් තිෙනවා.</v>
       </c>
       <c r="F29" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G29" t="str">
         <v>English Clipped Forms in Singlish; Isolated English Word Insertions in Singlish</v>
@@ -1177,10 +1167,10 @@
         <v>අද uni එකේ lec කියලා පෙනෙලා. මම lib එකේ sit කරන්නම් කියලා හිතුව ඒත් doc එකක් print කරන්නේ ගිය.</v>
       </c>
       <c r="E30" t="str">
-        <v/>
+        <v>අද uni එකේ lec කියලා පෙනෙලා. මම lib එකේ sit කරන්නම් කියලා හිතුව ඒත් doc එකක් print කරන්නේ ගිය.</v>
       </c>
       <c r="F30" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G30" t="str">
         <v>English Clipped Forms in Singlish; Isolated English Word Insertions in Singlish</v>
@@ -1203,10 +1193,10 @@
         <v>Galle යමුද අද?</v>
       </c>
       <c r="E31" t="str">
-        <v/>
+        <v>Galle යමුද අද?</v>
       </c>
       <c r="F31" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G31" t="str">
         <v>Place Names Embedded in Singlish; Question forms</v>
@@ -1229,10 +1219,10 @@
         <v>මම Nugegoda සිට Malabe යන්නේ ඕනේ. Kesbewa pass වෙනකොට call කරන්නම්. Boralesgamuwa hotel එකේ lunch කරන්නම්.</v>
       </c>
       <c r="E32" t="str">
-        <v/>
+        <v>මම Nugegoda සිට Malabe යන්නේ ඕනේ. Kesbewa pass වෙනකොට call කරන්නම්. Boralesgamuwa hotel එකේ lunch කරන්නම්.</v>
       </c>
       <c r="F32" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G32" t="str">
         <v>Place Names Embedded in Singlish; Isolated English Word Insertions in Singlish</v>
@@ -1255,10 +1245,10 @@
         <v>Ishara හෙට ආවාද?</v>
       </c>
       <c r="E33" t="str">
-        <v/>
+        <v>Ishara හෙට ආවාද?</v>
       </c>
       <c r="F33" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G33" t="str">
         <v>Person Names Embedded in Singlish; Question forms</v>
@@ -1281,10 +1271,10 @@
         <v>Kavindra සහ Thisara දෙන්නාම project එකේ work කරලා මාරු. ඒත් Dinusha කියනවා එහෙම නේ කියලා. ඔය Pavithra කියනවා ඒකා ගැනා?</v>
       </c>
       <c r="E34" t="str">
-        <v/>
+        <v>Kavindra සහ Thisara දෙන්නාම project එකේ work කරලා මාරු. ඒත් Dinusha කියනවා එහෙම නේ කියලා. ඔය Pavithra කියනවා ඒකා ගැනා?</v>
       </c>
       <c r="F34" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G34" t="str">
         <v>Person Names Embedded in Singlish; Isolated English Word Insertions in Singlish; Question forms</v>
@@ -1307,10 +1297,10 @@
         <v>2nd match එකේ score එකේ කියන්නේ.</v>
       </c>
       <c r="E35" t="str">
-        <v/>
+        <v>2nd match එකේ score එකේ කියන්නේ.</v>
       </c>
       <c r="F35" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G35" t="str">
         <v>Inputs with Numbers and Numeric Suffixes; Isolated English Word Insertions in Singlish</v>
@@ -1333,10 +1323,10 @@
         <v>science lab එකේ 1st group එකේ 98% අරගෙනේ. 2nd group එකේ 85k වාගේ markings. 3rd group වලට 50 සිට 75 දාකාවා.</v>
       </c>
       <c r="E36" t="str">
-        <v/>
+        <v>science lab එකේ 1st group එකේ 98% අරගෙනේ. 2nd group එකේ 85k වාගේ markings. 3rd group වලට 50 සිට 75 දාකාවා.</v>
       </c>
       <c r="F36" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G36" t="str">
         <v>Inputs with Numbers and Numeric Suffixes; English Clipped Forms in Singlish</v>
@@ -1359,10 +1349,10 @@
         <v>Rs. 1500 දෙන්නකෝ මචන්.</v>
       </c>
       <c r="E37" t="str">
-        <v/>
+        <v>Rs. 1500 දෙන්නකෝ මචන්.</v>
       </c>
       <c r="F37" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G37" t="str">
         <v>Inputs with Currency; Inputs with Slang and Casual Phrasing</v>
@@ -1385,10 +1375,10 @@
         <v>මම කිව්වා LKR 4500 වාගේ වේ යි කියලා. ඒත් USD 15 කියන්නේ රුපියල් වලින් කොච්චරද? EUR 100 කියන්නේ ගොඩක් නේ.</v>
       </c>
       <c r="E38" t="str">
-        <v/>
+        <v>මම කිව්වා LKR 4500 වාගේ වේ යි කියලා. ඒත් USD 15 කියන්නේ රුපියල් වලින් කොච්චරද? EUR 100 කියන්නේ ගොඩක් නේ.</v>
       </c>
       <c r="F38" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G38" t="str">
         <v>Inputs with Currency; Question forms</v>
@@ -1411,10 +1401,10 @@
         <v>4:30PM නාගින් එන්නේ කරන්නේ.</v>
       </c>
       <c r="E39" t="str">
-        <v/>
+        <v>4:30PM නාගින් එන්නේ කරන්නේ.</v>
       </c>
       <c r="F39" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G39" t="str">
         <v>Inputs with Time Formats; Command forms</v>
@@ -1437,10 +1427,10 @@
         <v>meeting එකේ 9:00AM වලට set කරනේ. මම 8:45 වලට එන්නේ හිතුව ඒත් traffic නිසා 9:15 වලට උනා. tomorrow 2:00PM වලට reschedule කරන්නම්.</v>
       </c>
       <c r="E40" t="str">
-        <v/>
+        <v>meeting එකේ 9:00AM වලට set කරනේ. මම 8:45 වලට එන්නේ හිතුව ඒත් traffic නිසා 9:15 වලට උනා. tomorrow 2:00PM වලට reschedule කරන්නම්.</v>
       </c>
       <c r="F40" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G40" t="str">
         <v>Inputs with Time Formats; Isolated English Word Insertions in Singlish</v>
@@ -1463,10 +1453,10 @@
         <v>2026-05-10 වලට submit කරන්නේ.</v>
       </c>
       <c r="E41" t="str">
-        <v/>
+        <v>2026-05-10 වලට submit කරන්නේ.</v>
       </c>
       <c r="F41" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G41" t="str">
         <v>Inputs with Dates; Isolated English Word Insertions in Singlish</v>
@@ -1489,10 +1479,10 @@
         <v>ඔය දන්නවා ද March 31 වෙනකොට deadline එකේ. මම April 1st වලට submit කරන්නම් කියලා හිතුව ඒත් April 5 වලට ඇහලා.</v>
       </c>
       <c r="E42" t="str">
-        <v/>
+        <v>ඔය දන්නවා ද March 31 වෙනකොට deadline එකේ. මම April 1st වලට submit කරන්නම් කියලා හිතුව ඒත් April 5 වලට ඇහලා.</v>
       </c>
       <c r="F42" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G42" t="str">
         <v>Inputs with Dates; Question forms; Inputs with Numbers and Numeric Suffixes</v>
@@ -1515,10 +1505,10 @@
         <v>kg 2ක් ගන්නවා නේ.</v>
       </c>
       <c r="E43" t="str">
-        <v/>
+        <v>kg 2ක් ගන්නවා නේ.</v>
       </c>
       <c r="F43" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G43" t="str">
         <v>Inputs with Unit of Measurements; Inputs with Numbers and Numeric Suffixes</v>
@@ -1541,10 +1531,10 @@
         <v>මම km 12ක් විතරේ යනේ. ඒ ගසේ උස මෙටෘ 8ක් විතරේ වේවා. ගෙදරේ සිට km 5 විතරේ ගිය.</v>
       </c>
       <c r="E44" t="str">
-        <v/>
+        <v>මම km 12ක් විතරේ යනේ. ඒ ගසේ උස මෙටෘ 8ක් විතරේ වේවා. ගෙදරේ සිට km 5 විතරේ ගිය.</v>
       </c>
       <c r="F44" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G44" t="str">
         <v>Inputs with Unit of Measurements; Inputs with Numbers and Numeric Suffixes</v>
@@ -1567,10 +1557,10 @@
         <v>බ්‍රෝ මාර කට්ටක් නේ උඹ.</v>
       </c>
       <c r="E45" t="str">
-        <v/>
+        <v>බ්රෝ මාර කට්ටක් නේ උඹ.</v>
       </c>
       <c r="F45" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G45" t="str">
         <v>Inputs with Slang and Casual Phrasing</v>
@@ -1593,10 +1583,10 @@
         <v>උඹ නිකන් ආකෙව් බලාමු කියලා. සිරාවට මෙකා එළකිරි set එකේ බ්‍රෝ. හොඳාටම set වෙලා තිෙනවා. අපේ gang එකේ හෙමෝම හදනවා.</v>
       </c>
       <c r="E46" t="str">
-        <v/>
+        <v>උඹ නිකන් ආකෙව් බලාමු කියලා. සිරාවට මෙකා එළකිරි set එකේ බ්රෝ. හොඳාටම set වෙලා තිෙනවා. අපේ gang එකේ හෙමෝම හදනවා.</v>
       </c>
       <c r="F46" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G46" t="str">
         <v>Inputs with Slang and Casual Phrasing; Isolated English Word Insertions in Singlish</v>
@@ -1619,10 +1609,10 @@
         <v>මේ link එකේ බලන්නේ: https://sinhala.wiki නේ. මම ඒකා පෙන්නන්නේ හිතුව.</v>
       </c>
       <c r="E47" t="str">
-        <v/>
+        <v>මේ link එකේ බලන්නේ: https://sinhala.wiki නේ. මම ඒකා පෙන්නන්නේ හිතුව.</v>
       </c>
       <c r="F47" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G47" t="str">
         <v>Online Identifiers in Singlish; English Digital Terms in Singlish</v>
@@ -1645,10 +1635,10 @@
         <v>මම email එකේ එවන්නේ: student.it23361522@university.lk කියලා දාන්නේ. @Nimal ඔයාට ඒකා send කරාද?</v>
       </c>
       <c r="E48" t="str">
-        <v/>
+        <v>මම email එකේ එවන්නේ: student.it23361522@university.lk කියලා දාන්නේ. @Nimal ඔයාට ඒකා send කරාද?</v>
       </c>
       <c r="F48" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G48" t="str">
         <v>Online Identifiers in Singlish; Person Names Embedded in Singlish; Question forms</v>
@@ -1671,10 +1661,10 @@
         <v>හොඳ වැඩේ කරලානේ 😊 බ්‍රෝ.</v>
       </c>
       <c r="E49" t="str">
-        <v/>
+        <v>හොඳ වැඩේ කරලානේ 😊 බ්රෝ.</v>
       </c>
       <c r="F49" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G49" t="str">
         <v>Inputs Containing Emojis; Inputs with Slang and Casual Phrasing</v>
@@ -1697,10 +1687,10 @@
         <v>අයියෝ මචන් 😢 මොකද වුනේ? මම කිව්වා නේ දෙන්නේ කියලා 😡 ඒත් ඔය ඒයාට දුන්නාද?</v>
       </c>
       <c r="E50" t="str">
-        <v/>
+        <v>අයියෝ මචන් 😢 මොකද වුනේ? මම කිව්වා නේ දෙන්නේ කියලා 😡 ඒත් ඔය ඒයාට දුන්නාද?</v>
       </c>
       <c r="F50" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G50" t="str">
         <v>Inputs Containing Emojis; Inputs with Slang and Casual Phrasing; Question forms</v>
@@ -1723,10 +1713,10 @@
         <v>මම අද office ආවේ පස්සේ Suresh ආවා ගෙදර. අපි කතා කළා 😊. මම කිව්වා "හෙට 9:00AM meeting එකක් තිෙනවා" කියලා. Suresh කිව්වා "ok මචන්, මම ASAP එන්නම්" කියලා. පස්සේ අපි Rs. 250 වාගේ බඩු කෑවා. මම කිව්වා March 20 exam කියලා calendar එකේ 2026-03-20 දාම්ම. ඒකා දුවස හදිස්සියේ ඒකා km 5ක් විතරේ පයින් යන්නේ උනා. 😄 හොඳ දිනයක්.</v>
       </c>
       <c r="E51" t="str">
-        <v/>
+        <v>මම අද office ආවේ පස්සේ Suresh ආවා ගෙදර. අපි කතා කළා 😊. මම කිව්වා "හෙට 9:00AM meeting එකක් තිෙනවා" කියලා. Suresh කිව්වා "ok මචන්, මම ASAP එන්නම්" කියලා. පස්සේ අපි Rs. 250 වාගේ බඩු කෑවා. මම කිව්වා March 20 exam කියලා calendar එකේ 2026-03-20 දාම්ම. ඒකා දුවස හදිස්සියේ ඒකා km 5ක් විතරේ පයින් යන්නේ උනා. 😄 හොඳ දිනයක්.</v>
       </c>
       <c r="F51" t="str">
-        <v/>
+        <v>Fail</v>
       </c>
       <c r="G51" t="str">
         <v>Inputs Containing Emojis; Person Names Embedded in Singlish; Inputs with Time Formats; Inputs with Currency; Inputs with Dates; Inputs with Unit of Measurements; English Abbreviations/Acronyms in Singlish; Isolated English Word Insertions in Singlish; Inputs with Slang and Casual Phrasing</v>

</xml_diff>